<commit_message>
Clean up project and improve UI styling
- Remove obsolete data files and old SEC downloads
- Clean up documentation and test files
- Enhance app.py UI with improved styling and formatting
- Update automated_sec_downloader.py
- Add Claude Code configuration

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEC_Excel_Downloads_AAPL_10-K/AAPL_10-K_Master_Consolidated_Financials_Detailed.xlsx
+++ b/SEC_Excel_Downloads_AAPL_10-K/AAPL_10-K_Master_Consolidated_Financials_Detailed.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN30"/>
+  <dimension ref="A1:X30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -456,22 +456,6 @@
     <col width="6" customWidth="1" min="22" max="22"/>
     <col width="6" customWidth="1" min="23" max="23"/>
     <col width="6" customWidth="1" min="24" max="24"/>
-    <col width="50" customWidth="1" min="25" max="25"/>
-    <col width="17" customWidth="1" min="26" max="26"/>
-    <col width="15" customWidth="1" min="27" max="27"/>
-    <col width="15" customWidth="1" min="28" max="28"/>
-    <col width="6" customWidth="1" min="29" max="29"/>
-    <col width="6" customWidth="1" min="30" max="30"/>
-    <col width="6" customWidth="1" min="31" max="31"/>
-    <col width="6" customWidth="1" min="32" max="32"/>
-    <col width="50" customWidth="1" min="33" max="33"/>
-    <col width="17" customWidth="1" min="34" max="34"/>
-    <col width="15" customWidth="1" min="35" max="35"/>
-    <col width="15" customWidth="1" min="36" max="36"/>
-    <col width="6" customWidth="1" min="37" max="37"/>
-    <col width="6" customWidth="1" min="38" max="38"/>
-    <col width="6" customWidth="1" min="39" max="39"/>
-    <col width="6" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,16 +482,6 @@
           <t>Year 2022</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>Year 2021</t>
-        </is>
-      </c>
-      <c r="AG3" s="2" t="inlineStr">
-        <is>
-          <t>Year 2020</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -525,16 +499,6 @@
           <t>Income Statement</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Income Statement</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>Income Statement</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -567,26 +531,6 @@
           <t>12 Months Ended</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED STATEMENTS OF OPERATIONS - USD ($) shares in Thousands, $ in Millions</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>12 Months Ended</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED STATEMENTS OF OPERATIONS - USD ($) shares in Thousands, $ in Millions</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>12 Months Ended</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -634,36 +578,6 @@
           <t>Sep. 26, 2020</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>Sep. 25, 2021</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>Sep. 26, 2020</t>
-        </is>
-      </c>
-      <c r="AB6" t="inlineStr">
-        <is>
-          <t>Sep. 28, 2019</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>Sep. 26, 2020</t>
-        </is>
-      </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>Sep. 28, 2019</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>Sep. 29, 2018</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -708,34 +622,6 @@
       <c r="T7" s="3" t="n">
         <v>274515</v>
       </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>Net sales</t>
-        </is>
-      </c>
-      <c r="Z7" s="3" t="n">
-        <v>365817</v>
-      </c>
-      <c r="AA7" s="3" t="n">
-        <v>274515</v>
-      </c>
-      <c r="AB7" s="3" t="n">
-        <v>260174</v>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>Net sales</t>
-        </is>
-      </c>
-      <c r="AH7" s="3" t="n">
-        <v>274515</v>
-      </c>
-      <c r="AI7" s="3" t="n">
-        <v>260174</v>
-      </c>
-      <c r="AJ7" s="3" t="n">
-        <v>265595</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -780,34 +666,6 @@
       <c r="T8" s="3" t="n">
         <v>169559</v>
       </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>Cost of sales</t>
-        </is>
-      </c>
-      <c r="Z8" s="3" t="n">
-        <v>212981</v>
-      </c>
-      <c r="AA8" s="3" t="n">
-        <v>169559</v>
-      </c>
-      <c r="AB8" s="3" t="n">
-        <v>161782</v>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>Cost of sales</t>
-        </is>
-      </c>
-      <c r="AH8" s="3" t="n">
-        <v>169559</v>
-      </c>
-      <c r="AI8" s="3" t="n">
-        <v>161782</v>
-      </c>
-      <c r="AJ8" s="3" t="n">
-        <v>163756</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -852,34 +710,6 @@
       <c r="T9" s="3" t="n">
         <v>104956</v>
       </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>Gross margin</t>
-        </is>
-      </c>
-      <c r="Z9" s="3" t="n">
-        <v>152836</v>
-      </c>
-      <c r="AA9" s="3" t="n">
-        <v>104956</v>
-      </c>
-      <c r="AB9" s="3" t="n">
-        <v>98392</v>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>Gross margin</t>
-        </is>
-      </c>
-      <c r="AH9" s="3" t="n">
-        <v>104956</v>
-      </c>
-      <c r="AI9" s="3" t="n">
-        <v>98392</v>
-      </c>
-      <c r="AJ9" s="3" t="n">
-        <v>101839</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -942,16 +772,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>Operating expenses:</t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>Operating expenses:</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -996,34 +816,6 @@
       <c r="T11" s="3" t="n">
         <v>18752</v>
       </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Research and development</t>
-        </is>
-      </c>
-      <c r="Z11" s="3" t="n">
-        <v>21914</v>
-      </c>
-      <c r="AA11" s="3" t="n">
-        <v>18752</v>
-      </c>
-      <c r="AB11" s="3" t="n">
-        <v>16217</v>
-      </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>Research and development</t>
-        </is>
-      </c>
-      <c r="AH11" s="3" t="n">
-        <v>18752</v>
-      </c>
-      <c r="AI11" s="3" t="n">
-        <v>16217</v>
-      </c>
-      <c r="AJ11" s="3" t="n">
-        <v>14236</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1068,34 +860,6 @@
       <c r="T12" s="3" t="n">
         <v>19916</v>
       </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>Selling, general and administrative</t>
-        </is>
-      </c>
-      <c r="Z12" s="3" t="n">
-        <v>21973</v>
-      </c>
-      <c r="AA12" s="3" t="n">
-        <v>19916</v>
-      </c>
-      <c r="AB12" s="3" t="n">
-        <v>18245</v>
-      </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>Selling, general and administrative</t>
-        </is>
-      </c>
-      <c r="AH12" s="3" t="n">
-        <v>19916</v>
-      </c>
-      <c r="AI12" s="3" t="n">
-        <v>18245</v>
-      </c>
-      <c r="AJ12" s="3" t="n">
-        <v>16705</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1140,34 +904,6 @@
       <c r="T13" s="3" t="n">
         <v>38668</v>
       </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>Total operating expenses</t>
-        </is>
-      </c>
-      <c r="Z13" s="3" t="n">
-        <v>43887</v>
-      </c>
-      <c r="AA13" s="3" t="n">
-        <v>38668</v>
-      </c>
-      <c r="AB13" s="3" t="n">
-        <v>34462</v>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>Total operating expenses</t>
-        </is>
-      </c>
-      <c r="AH13" s="3" t="n">
-        <v>38668</v>
-      </c>
-      <c r="AI13" s="3" t="n">
-        <v>34462</v>
-      </c>
-      <c r="AJ13" s="3" t="n">
-        <v>30941</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1212,34 +948,6 @@
       <c r="T14" s="3" t="n">
         <v>66288</v>
       </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>Operating income</t>
-        </is>
-      </c>
-      <c r="Z14" s="3" t="n">
-        <v>108949</v>
-      </c>
-      <c r="AA14" s="3" t="n">
-        <v>66288</v>
-      </c>
-      <c r="AB14" s="3" t="n">
-        <v>63930</v>
-      </c>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>Operating income</t>
-        </is>
-      </c>
-      <c r="AH14" s="3" t="n">
-        <v>66288</v>
-      </c>
-      <c r="AI14" s="3" t="n">
-        <v>63930</v>
-      </c>
-      <c r="AJ14" s="3" t="n">
-        <v>70898</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1284,34 +992,6 @@
       <c r="T15" s="4" t="n">
         <v>803</v>
       </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>Other income/(expense), net</t>
-        </is>
-      </c>
-      <c r="Z15" s="4" t="n">
-        <v>258</v>
-      </c>
-      <c r="AA15" s="4" t="n">
-        <v>803</v>
-      </c>
-      <c r="AB15" s="3" t="n">
-        <v>1807</v>
-      </c>
-      <c r="AG15" t="inlineStr">
-        <is>
-          <t>Other income/(expense), net</t>
-        </is>
-      </c>
-      <c r="AH15" s="4" t="n">
-        <v>803</v>
-      </c>
-      <c r="AI15" s="3" t="n">
-        <v>1807</v>
-      </c>
-      <c r="AJ15" s="3" t="n">
-        <v>2005</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1356,34 +1036,6 @@
       <c r="T16" s="3" t="n">
         <v>67091</v>
       </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>Income before provision for income taxes</t>
-        </is>
-      </c>
-      <c r="Z16" s="3" t="n">
-        <v>109207</v>
-      </c>
-      <c r="AA16" s="3" t="n">
-        <v>67091</v>
-      </c>
-      <c r="AB16" s="3" t="n">
-        <v>65737</v>
-      </c>
-      <c r="AG16" t="inlineStr">
-        <is>
-          <t>Income before provision for income taxes</t>
-        </is>
-      </c>
-      <c r="AH16" s="3" t="n">
-        <v>67091</v>
-      </c>
-      <c r="AI16" s="3" t="n">
-        <v>65737</v>
-      </c>
-      <c r="AJ16" s="3" t="n">
-        <v>72903</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1428,34 +1080,6 @@
       <c r="T17" s="3" t="n">
         <v>9680</v>
       </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>Provision for income taxes</t>
-        </is>
-      </c>
-      <c r="Z17" s="3" t="n">
-        <v>14527</v>
-      </c>
-      <c r="AA17" s="3" t="n">
-        <v>9680</v>
-      </c>
-      <c r="AB17" s="3" t="n">
-        <v>10481</v>
-      </c>
-      <c r="AG17" t="inlineStr">
-        <is>
-          <t>Provision for income taxes</t>
-        </is>
-      </c>
-      <c r="AH17" s="3" t="n">
-        <v>9680</v>
-      </c>
-      <c r="AI17" s="3" t="n">
-        <v>10481</v>
-      </c>
-      <c r="AJ17" s="3" t="n">
-        <v>13372</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1500,34 +1124,6 @@
       <c r="T18" s="3" t="n">
         <v>57411</v>
       </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>Net income</t>
-        </is>
-      </c>
-      <c r="Z18" s="3" t="n">
-        <v>94680</v>
-      </c>
-      <c r="AA18" s="3" t="n">
-        <v>57411</v>
-      </c>
-      <c r="AB18" s="3" t="n">
-        <v>55256</v>
-      </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>Net income</t>
-        </is>
-      </c>
-      <c r="AH18" s="3" t="n">
-        <v>57411</v>
-      </c>
-      <c r="AI18" s="3" t="n">
-        <v>55256</v>
-      </c>
-      <c r="AJ18" s="3" t="n">
-        <v>59531</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1590,16 +1186,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>Earnings per share:</t>
-        </is>
-      </c>
-      <c r="AG19" t="inlineStr">
-        <is>
-          <t>Earnings per share:</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1644,34 +1230,6 @@
       <c r="T20" s="4" t="n">
         <v>3.31</v>
       </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>Basic (in dollars per share)</t>
-        </is>
-      </c>
-      <c r="Z20" s="4" t="n">
-        <v>5.67</v>
-      </c>
-      <c r="AA20" s="4" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="AB20" s="4" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="AG20" t="inlineStr">
-        <is>
-          <t>Basic (in dollars per share)</t>
-        </is>
-      </c>
-      <c r="AH20" s="4" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="AI20" s="4" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="AJ20" s="4" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1716,34 +1274,6 @@
       <c r="T21" s="4" t="n">
         <v>3.28</v>
       </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>Diluted (in dollars per share)</t>
-        </is>
-      </c>
-      <c r="Z21" s="4" t="n">
-        <v>5.61</v>
-      </c>
-      <c r="AA21" s="4" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="AB21" s="4" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="AG21" t="inlineStr">
-        <is>
-          <t>Diluted (in dollars per share)</t>
-        </is>
-      </c>
-      <c r="AH21" s="4" t="n">
-        <v>3.28</v>
-      </c>
-      <c r="AI21" s="4" t="n">
-        <v>2.97</v>
-      </c>
-      <c r="AJ21" s="4" t="n">
-        <v>2.98</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1806,16 +1336,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>Shares used in computing earnings per share:</t>
-        </is>
-      </c>
-      <c r="AG22" t="inlineStr">
-        <is>
-          <t>Shares used in computing earnings per share:</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1860,34 +1380,6 @@
       <c r="T23" s="3" t="n">
         <v>17352119</v>
       </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>Basic (in shares)</t>
-        </is>
-      </c>
-      <c r="Z23" s="3" t="n">
-        <v>16701272</v>
-      </c>
-      <c r="AA23" s="3" t="n">
-        <v>17352119</v>
-      </c>
-      <c r="AB23" s="3" t="n">
-        <v>18471336</v>
-      </c>
-      <c r="AG23" t="inlineStr">
-        <is>
-          <t>Basic (in shares)</t>
-        </is>
-      </c>
-      <c r="AH23" s="3" t="n">
-        <v>17352119</v>
-      </c>
-      <c r="AI23" s="3" t="n">
-        <v>18471336</v>
-      </c>
-      <c r="AJ23" s="3" t="n">
-        <v>19821510</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1932,34 +1424,6 @@
       <c r="T24" s="3" t="n">
         <v>17528214</v>
       </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>Diluted (in shares)</t>
-        </is>
-      </c>
-      <c r="Z24" s="3" t="n">
-        <v>16864919</v>
-      </c>
-      <c r="AA24" s="3" t="n">
-        <v>17528214</v>
-      </c>
-      <c r="AB24" s="3" t="n">
-        <v>18595651</v>
-      </c>
-      <c r="AG24" t="inlineStr">
-        <is>
-          <t>Diluted (in shares)</t>
-        </is>
-      </c>
-      <c r="AH24" s="3" t="n">
-        <v>17528214</v>
-      </c>
-      <c r="AI24" s="3" t="n">
-        <v>18595651</v>
-      </c>
-      <c r="AJ24" s="3" t="n">
-        <v>20000435</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2022,16 +1486,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
-      <c r="AG25" t="inlineStr">
-        <is>
-          <t>Products</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2076,34 +1530,6 @@
       <c r="T26" s="3" t="n">
         <v>220747</v>
       </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>Net sales</t>
-        </is>
-      </c>
-      <c r="Z26" s="3" t="n">
-        <v>297392</v>
-      </c>
-      <c r="AA26" s="3" t="n">
-        <v>220747</v>
-      </c>
-      <c r="AB26" s="3" t="n">
-        <v>213883</v>
-      </c>
-      <c r="AG26" t="inlineStr">
-        <is>
-          <t>Net sales</t>
-        </is>
-      </c>
-      <c r="AH26" s="3" t="n">
-        <v>220747</v>
-      </c>
-      <c r="AI26" s="3" t="n">
-        <v>213883</v>
-      </c>
-      <c r="AJ26" s="3" t="n">
-        <v>225847</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2148,34 +1574,6 @@
       <c r="T27" s="3" t="n">
         <v>151286</v>
       </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>Cost of sales</t>
-        </is>
-      </c>
-      <c r="Z27" s="3" t="n">
-        <v>192266</v>
-      </c>
-      <c r="AA27" s="3" t="n">
-        <v>151286</v>
-      </c>
-      <c r="AB27" s="3" t="n">
-        <v>144996</v>
-      </c>
-      <c r="AG27" t="inlineStr">
-        <is>
-          <t>Cost of sales</t>
-        </is>
-      </c>
-      <c r="AH27" s="3" t="n">
-        <v>151286</v>
-      </c>
-      <c r="AI27" s="3" t="n">
-        <v>144996</v>
-      </c>
-      <c r="AJ27" s="3" t="n">
-        <v>148164</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2238,16 +1636,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>Services</t>
-        </is>
-      </c>
-      <c r="AG28" t="inlineStr">
-        <is>
-          <t>Services</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2292,34 +1680,6 @@
       <c r="T29" s="3" t="n">
         <v>53768</v>
       </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>Net sales</t>
-        </is>
-      </c>
-      <c r="Z29" s="3" t="n">
-        <v>68425</v>
-      </c>
-      <c r="AA29" s="3" t="n">
-        <v>53768</v>
-      </c>
-      <c r="AB29" s="3" t="n">
-        <v>46291</v>
-      </c>
-      <c r="AG29" t="inlineStr">
-        <is>
-          <t>Net sales</t>
-        </is>
-      </c>
-      <c r="AH29" s="3" t="n">
-        <v>53768</v>
-      </c>
-      <c r="AI29" s="3" t="n">
-        <v>46291</v>
-      </c>
-      <c r="AJ29" s="3" t="n">
-        <v>39748</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2364,42 +1724,12 @@
       <c r="T30" s="3" t="n">
         <v>18273</v>
       </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>Cost of sales</t>
-        </is>
-      </c>
-      <c r="Z30" s="3" t="n">
-        <v>20715</v>
-      </c>
-      <c r="AA30" s="3" t="n">
-        <v>18273</v>
-      </c>
-      <c r="AB30" s="3" t="n">
-        <v>16786</v>
-      </c>
-      <c r="AG30" t="inlineStr">
-        <is>
-          <t>Cost of sales</t>
-        </is>
-      </c>
-      <c r="AH30" s="3" t="n">
-        <v>18273</v>
-      </c>
-      <c r="AI30" s="3" t="n">
-        <v>16786</v>
-      </c>
-      <c r="AJ30" s="3" t="n">
-        <v>15592</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="AG3:AN3"/>
     <mergeCell ref="Q3:X3"/>
     <mergeCell ref="I3:P3"/>
-    <mergeCell ref="Y3:AF3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2411,7 +1741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN41"/>
+  <dimension ref="A1:X41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2438,22 +1768,6 @@
     <col width="6" customWidth="1" min="22" max="22"/>
     <col width="6" customWidth="1" min="23" max="23"/>
     <col width="6" customWidth="1" min="24" max="24"/>
-    <col width="50" customWidth="1" min="25" max="25"/>
-    <col width="15" customWidth="1" min="26" max="26"/>
-    <col width="15" customWidth="1" min="27" max="27"/>
-    <col width="6" customWidth="1" min="28" max="28"/>
-    <col width="6" customWidth="1" min="29" max="29"/>
-    <col width="6" customWidth="1" min="30" max="30"/>
-    <col width="6" customWidth="1" min="31" max="31"/>
-    <col width="6" customWidth="1" min="32" max="32"/>
-    <col width="50" customWidth="1" min="33" max="33"/>
-    <col width="15" customWidth="1" min="34" max="34"/>
-    <col width="15" customWidth="1" min="35" max="35"/>
-    <col width="6" customWidth="1" min="36" max="36"/>
-    <col width="6" customWidth="1" min="37" max="37"/>
-    <col width="6" customWidth="1" min="38" max="38"/>
-    <col width="6" customWidth="1" min="39" max="39"/>
-    <col width="6" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2480,16 +1794,6 @@
           <t>Year 2022</t>
         </is>
       </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>Year 2021</t>
-        </is>
-      </c>
-      <c r="AG3" s="2" t="inlineStr">
-        <is>
-          <t>Year 2020</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2507,16 +1811,6 @@
           <t>Balance Sheet</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Balance Sheet</t>
-        </is>
-      </c>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>Balance Sheet</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2564,36 +1858,6 @@
           <t>Sep. 25, 2021</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED BALANCE SHEETS - USD ($) $ in Millions</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>Sep. 25, 2021</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>Sep. 26, 2020</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED BALANCE SHEETS - USD ($) $ in Millions</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>Sep. 26, 2020</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>Sep. 28, 2019</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2641,16 +1905,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>Current assets:</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>Current assets:</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2686,28 +1940,6 @@
       <c r="S7" s="3" t="n">
         <v>34940</v>
       </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>Cash and cash equivalents</t>
-        </is>
-      </c>
-      <c r="Z7" s="3" t="n">
-        <v>34940</v>
-      </c>
-      <c r="AA7" s="3" t="n">
-        <v>38016</v>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>Cash and cash equivalents</t>
-        </is>
-      </c>
-      <c r="AH7" s="3" t="n">
-        <v>38016</v>
-      </c>
-      <c r="AI7" s="3" t="n">
-        <v>48844</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2743,28 +1975,6 @@
       <c r="S8" s="3" t="n">
         <v>27699</v>
       </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>Marketable securities</t>
-        </is>
-      </c>
-      <c r="Z8" s="3" t="n">
-        <v>27699</v>
-      </c>
-      <c r="AA8" s="3" t="n">
-        <v>52927</v>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>Marketable securities</t>
-        </is>
-      </c>
-      <c r="AH8" s="3" t="n">
-        <v>52927</v>
-      </c>
-      <c r="AI8" s="3" t="n">
-        <v>51713</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2800,28 +2010,6 @@
       <c r="S9" s="3" t="n">
         <v>26278</v>
       </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>Accounts receivable, net</t>
-        </is>
-      </c>
-      <c r="Z9" s="3" t="n">
-        <v>26278</v>
-      </c>
-      <c r="AA9" s="3" t="n">
-        <v>16120</v>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>Accounts receivable, net</t>
-        </is>
-      </c>
-      <c r="AH9" s="3" t="n">
-        <v>16120</v>
-      </c>
-      <c r="AI9" s="3" t="n">
-        <v>22926</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2857,28 +2045,6 @@
       <c r="S10" s="3" t="n">
         <v>6580</v>
       </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>Inventories</t>
-        </is>
-      </c>
-      <c r="Z10" s="3" t="n">
-        <v>6580</v>
-      </c>
-      <c r="AA10" s="3" t="n">
-        <v>4061</v>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>Inventories</t>
-        </is>
-      </c>
-      <c r="AH10" s="3" t="n">
-        <v>4061</v>
-      </c>
-      <c r="AI10" s="3" t="n">
-        <v>4106</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2914,28 +2080,6 @@
       <c r="S11" s="3" t="n">
         <v>25228</v>
       </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Vendor non-trade receivables</t>
-        </is>
-      </c>
-      <c r="Z11" s="3" t="n">
-        <v>25228</v>
-      </c>
-      <c r="AA11" s="3" t="n">
-        <v>21325</v>
-      </c>
-      <c r="AG11" t="inlineStr">
-        <is>
-          <t>Vendor non-trade receivables</t>
-        </is>
-      </c>
-      <c r="AH11" s="3" t="n">
-        <v>21325</v>
-      </c>
-      <c r="AI11" s="3" t="n">
-        <v>22878</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2971,28 +2115,6 @@
       <c r="S12" s="3" t="n">
         <v>14111</v>
       </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>Other current assets</t>
-        </is>
-      </c>
-      <c r="Z12" s="3" t="n">
-        <v>14111</v>
-      </c>
-      <c r="AA12" s="3" t="n">
-        <v>11264</v>
-      </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>Other current assets</t>
-        </is>
-      </c>
-      <c r="AH12" s="3" t="n">
-        <v>11264</v>
-      </c>
-      <c r="AI12" s="3" t="n">
-        <v>12352</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3028,28 +2150,6 @@
       <c r="S13" s="3" t="n">
         <v>134836</v>
       </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>Total current assets</t>
-        </is>
-      </c>
-      <c r="Z13" s="3" t="n">
-        <v>134836</v>
-      </c>
-      <c r="AA13" s="3" t="n">
-        <v>143713</v>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>Total current assets</t>
-        </is>
-      </c>
-      <c r="AH13" s="3" t="n">
-        <v>143713</v>
-      </c>
-      <c r="AI13" s="3" t="n">
-        <v>162819</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3097,16 +2197,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>Non-current assets:</t>
-        </is>
-      </c>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>Non-current assets:</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3142,28 +2232,6 @@
       <c r="S15" s="3" t="n">
         <v>127877</v>
       </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>Marketable securities</t>
-        </is>
-      </c>
-      <c r="Z15" s="3" t="n">
-        <v>127877</v>
-      </c>
-      <c r="AA15" s="3" t="n">
-        <v>100887</v>
-      </c>
-      <c r="AG15" t="inlineStr">
-        <is>
-          <t>Marketable securities</t>
-        </is>
-      </c>
-      <c r="AH15" s="3" t="n">
-        <v>100887</v>
-      </c>
-      <c r="AI15" s="3" t="n">
-        <v>105341</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3199,28 +2267,6 @@
       <c r="S16" s="3" t="n">
         <v>39440</v>
       </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>Property, plant and equipment, net</t>
-        </is>
-      </c>
-      <c r="Z16" s="3" t="n">
-        <v>39440</v>
-      </c>
-      <c r="AA16" s="3" t="n">
-        <v>36766</v>
-      </c>
-      <c r="AG16" t="inlineStr">
-        <is>
-          <t>Property, plant and equipment, net</t>
-        </is>
-      </c>
-      <c r="AH16" s="3" t="n">
-        <v>36766</v>
-      </c>
-      <c r="AI16" s="3" t="n">
-        <v>37378</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3256,28 +2302,6 @@
       <c r="S17" s="3" t="n">
         <v>48849</v>
       </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>Other non-current assets</t>
-        </is>
-      </c>
-      <c r="Z17" s="3" t="n">
-        <v>48849</v>
-      </c>
-      <c r="AA17" s="3" t="n">
-        <v>42522</v>
-      </c>
-      <c r="AG17" t="inlineStr">
-        <is>
-          <t>Other non-current assets</t>
-        </is>
-      </c>
-      <c r="AH17" s="3" t="n">
-        <v>42522</v>
-      </c>
-      <c r="AI17" s="3" t="n">
-        <v>32978</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3313,28 +2337,6 @@
       <c r="S18" s="3" t="n">
         <v>216166</v>
       </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>Total non-current assets</t>
-        </is>
-      </c>
-      <c r="Z18" s="3" t="n">
-        <v>216166</v>
-      </c>
-      <c r="AA18" s="3" t="n">
-        <v>180175</v>
-      </c>
-      <c r="AG18" t="inlineStr">
-        <is>
-          <t>Total non-current assets</t>
-        </is>
-      </c>
-      <c r="AH18" s="3" t="n">
-        <v>180175</v>
-      </c>
-      <c r="AI18" s="3" t="n">
-        <v>175697</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3370,28 +2372,6 @@
       <c r="S19" s="3" t="n">
         <v>351002</v>
       </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>Total assets</t>
-        </is>
-      </c>
-      <c r="Z19" s="3" t="n">
-        <v>351002</v>
-      </c>
-      <c r="AA19" s="3" t="n">
-        <v>323888</v>
-      </c>
-      <c r="AG19" t="inlineStr">
-        <is>
-          <t>Total assets</t>
-        </is>
-      </c>
-      <c r="AH19" s="3" t="n">
-        <v>323888</v>
-      </c>
-      <c r="AI19" s="3" t="n">
-        <v>338516</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3439,16 +2419,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>Current liabilities:</t>
-        </is>
-      </c>
-      <c r="AG20" t="inlineStr">
-        <is>
-          <t>Current liabilities:</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3484,28 +2454,6 @@
       <c r="S21" s="3" t="n">
         <v>54763</v>
       </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>Accounts payable</t>
-        </is>
-      </c>
-      <c r="Z21" s="3" t="n">
-        <v>54763</v>
-      </c>
-      <c r="AA21" s="3" t="n">
-        <v>42296</v>
-      </c>
-      <c r="AG21" t="inlineStr">
-        <is>
-          <t>Accounts payable</t>
-        </is>
-      </c>
-      <c r="AH21" s="3" t="n">
-        <v>42296</v>
-      </c>
-      <c r="AI21" s="3" t="n">
-        <v>46236</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3541,28 +2489,6 @@
       <c r="S22" s="3" t="n">
         <v>47493</v>
       </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>Other current liabilities</t>
-        </is>
-      </c>
-      <c r="Z22" s="3" t="n">
-        <v>47493</v>
-      </c>
-      <c r="AA22" s="3" t="n">
-        <v>42684</v>
-      </c>
-      <c r="AG22" t="inlineStr">
-        <is>
-          <t>Other current liabilities</t>
-        </is>
-      </c>
-      <c r="AH22" s="3" t="n">
-        <v>42684</v>
-      </c>
-      <c r="AI22" s="3" t="n">
-        <v>37720</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3598,28 +2524,6 @@
       <c r="S23" s="3" t="n">
         <v>7612</v>
       </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>Deferred revenue</t>
-        </is>
-      </c>
-      <c r="Z23" s="3" t="n">
-        <v>7612</v>
-      </c>
-      <c r="AA23" s="3" t="n">
-        <v>6643</v>
-      </c>
-      <c r="AG23" t="inlineStr">
-        <is>
-          <t>Deferred revenue</t>
-        </is>
-      </c>
-      <c r="AH23" s="3" t="n">
-        <v>6643</v>
-      </c>
-      <c r="AI23" s="3" t="n">
-        <v>5522</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3655,28 +2559,6 @@
       <c r="S24" s="3" t="n">
         <v>6000</v>
       </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>Commercial paper</t>
-        </is>
-      </c>
-      <c r="Z24" s="3" t="n">
-        <v>6000</v>
-      </c>
-      <c r="AA24" s="3" t="n">
-        <v>4996</v>
-      </c>
-      <c r="AG24" t="inlineStr">
-        <is>
-          <t>Commercial paper</t>
-        </is>
-      </c>
-      <c r="AH24" s="3" t="n">
-        <v>4996</v>
-      </c>
-      <c r="AI24" s="3" t="n">
-        <v>5980</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3712,28 +2594,6 @@
       <c r="S25" s="3" t="n">
         <v>9613</v>
       </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>Term debt</t>
-        </is>
-      </c>
-      <c r="Z25" s="3" t="n">
-        <v>9613</v>
-      </c>
-      <c r="AA25" s="3" t="n">
-        <v>8773</v>
-      </c>
-      <c r="AG25" t="inlineStr">
-        <is>
-          <t>Term debt</t>
-        </is>
-      </c>
-      <c r="AH25" s="3" t="n">
-        <v>8773</v>
-      </c>
-      <c r="AI25" s="3" t="n">
-        <v>10260</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3769,28 +2629,6 @@
       <c r="S26" s="3" t="n">
         <v>125481</v>
       </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>Total current liabilities</t>
-        </is>
-      </c>
-      <c r="Z26" s="3" t="n">
-        <v>125481</v>
-      </c>
-      <c r="AA26" s="3" t="n">
-        <v>105392</v>
-      </c>
-      <c r="AG26" t="inlineStr">
-        <is>
-          <t>Total current liabilities</t>
-        </is>
-      </c>
-      <c r="AH26" s="3" t="n">
-        <v>105392</v>
-      </c>
-      <c r="AI26" s="3" t="n">
-        <v>105718</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3838,16 +2676,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>Non-current liabilities:</t>
-        </is>
-      </c>
-      <c r="AG27" t="inlineStr">
-        <is>
-          <t>Non-current liabilities:</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3883,28 +2711,6 @@
       <c r="S28" s="3" t="n">
         <v>109106</v>
       </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>Term debt</t>
-        </is>
-      </c>
-      <c r="Z28" s="3" t="n">
-        <v>109106</v>
-      </c>
-      <c r="AA28" s="3" t="n">
-        <v>98667</v>
-      </c>
-      <c r="AG28" t="inlineStr">
-        <is>
-          <t>Term debt</t>
-        </is>
-      </c>
-      <c r="AH28" s="3" t="n">
-        <v>98667</v>
-      </c>
-      <c r="AI28" s="3" t="n">
-        <v>91807</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3940,28 +2746,6 @@
       <c r="S29" s="3" t="n">
         <v>53325</v>
       </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>Other non-current liabilities</t>
-        </is>
-      </c>
-      <c r="Z29" s="3" t="n">
-        <v>53325</v>
-      </c>
-      <c r="AA29" s="3" t="n">
-        <v>54490</v>
-      </c>
-      <c r="AG29" t="inlineStr">
-        <is>
-          <t>Other non-current liabilities</t>
-        </is>
-      </c>
-      <c r="AH29" s="3" t="n">
-        <v>54490</v>
-      </c>
-      <c r="AI29" s="3" t="n">
-        <v>50503</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3997,28 +2781,6 @@
       <c r="S30" s="3" t="n">
         <v>162431</v>
       </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>Total non-current liabilities</t>
-        </is>
-      </c>
-      <c r="Z30" s="3" t="n">
-        <v>162431</v>
-      </c>
-      <c r="AA30" s="3" t="n">
-        <v>153157</v>
-      </c>
-      <c r="AG30" t="inlineStr">
-        <is>
-          <t>Total non-current liabilities</t>
-        </is>
-      </c>
-      <c r="AH30" s="3" t="n">
-        <v>153157</v>
-      </c>
-      <c r="AI30" s="3" t="n">
-        <v>142310</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4054,28 +2816,6 @@
       <c r="S31" s="3" t="n">
         <v>287912</v>
       </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>Total liabilities</t>
-        </is>
-      </c>
-      <c r="Z31" s="3" t="n">
-        <v>287912</v>
-      </c>
-      <c r="AA31" s="3" t="n">
-        <v>258549</v>
-      </c>
-      <c r="AG31" t="inlineStr">
-        <is>
-          <t>Total liabilities</t>
-        </is>
-      </c>
-      <c r="AH31" s="3" t="n">
-        <v>258549</v>
-      </c>
-      <c r="AI31" s="3" t="n">
-        <v>248028</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4123,36 +2863,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>Commitments and contingencies</t>
-        </is>
-      </c>
-      <c r="Z32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AG32" t="inlineStr">
-        <is>
-          <t>Commitments and contingencies</t>
-        </is>
-      </c>
-      <c r="AH32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
-      <c r="AI32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> </t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4192,16 +2902,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="Y33" t="inlineStr">
-        <is>
-          <t>Shareholders’ equity:</t>
-        </is>
-      </c>
-      <c r="AG33" t="inlineStr">
-        <is>
-          <t>Shareholders’ equity:</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4237,28 +2937,6 @@
       <c r="S34" s="3" t="n">
         <v>57365</v>
       </c>
-      <c r="Y34" t="inlineStr">
-        <is>
-          <t>Common stock and additional paid-in capital, $0.00001 par value: 50,400,000 shares authorized; 16,426,786 and 16,976,763 shares issued and outstanding, respectively</t>
-        </is>
-      </c>
-      <c r="Z34" s="3" t="n">
-        <v>57365</v>
-      </c>
-      <c r="AA34" s="3" t="n">
-        <v>50779</v>
-      </c>
-      <c r="AG34" t="inlineStr">
-        <is>
-          <t>Common stock and additional paid-in capital, $0.00001 par value: 50,400,000 shares authorized; 16,976,763 and 17,772,945 shares issued and outstanding, respectively</t>
-        </is>
-      </c>
-      <c r="AH34" s="3" t="n">
-        <v>50779</v>
-      </c>
-      <c r="AI34" s="3" t="n">
-        <v>45174</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4302,28 +2980,6 @@
       <c r="S35" s="3" t="n">
         <v>5562</v>
       </c>
-      <c r="Y35" t="inlineStr">
-        <is>
-          <t>Retained earnings</t>
-        </is>
-      </c>
-      <c r="Z35" s="3" t="n">
-        <v>5562</v>
-      </c>
-      <c r="AA35" s="3" t="n">
-        <v>14966</v>
-      </c>
-      <c r="AG35" t="inlineStr">
-        <is>
-          <t>Retained earnings</t>
-        </is>
-      </c>
-      <c r="AH35" s="3" t="n">
-        <v>14966</v>
-      </c>
-      <c r="AI35" s="3" t="n">
-        <v>45898</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4359,28 +3015,6 @@
       <c r="S36" s="4" t="n">
         <v>163</v>
       </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>Accumulated other comprehensive income/(loss)</t>
-        </is>
-      </c>
-      <c r="Z36" s="4" t="n">
-        <v>163</v>
-      </c>
-      <c r="AA36" s="4" t="n">
-        <v>-406</v>
-      </c>
-      <c r="AG36" t="inlineStr">
-        <is>
-          <t>Accumulated other comprehensive income/(loss)</t>
-        </is>
-      </c>
-      <c r="AH36" s="4" t="n">
-        <v>-406</v>
-      </c>
-      <c r="AI36" s="4" t="n">
-        <v>-584</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4416,28 +3050,6 @@
       <c r="S37" s="3" t="n">
         <v>63090</v>
       </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>Total shareholders’ equity</t>
-        </is>
-      </c>
-      <c r="Z37" s="3" t="n">
-        <v>63090</v>
-      </c>
-      <c r="AA37" s="3" t="n">
-        <v>65339</v>
-      </c>
-      <c r="AG37" t="inlineStr">
-        <is>
-          <t>Total shareholders’ equity</t>
-        </is>
-      </c>
-      <c r="AH37" s="3" t="n">
-        <v>65339</v>
-      </c>
-      <c r="AI37" s="3" t="n">
-        <v>90488</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4473,28 +3085,6 @@
       <c r="S38" s="3" t="n">
         <v>351002</v>
       </c>
-      <c r="Y38" t="inlineStr">
-        <is>
-          <t>Total liabilities and shareholders’ equity</t>
-        </is>
-      </c>
-      <c r="Z38" s="3" t="n">
-        <v>351002</v>
-      </c>
-      <c r="AA38" s="3" t="n">
-        <v>323888</v>
-      </c>
-      <c r="AG38" t="inlineStr">
-        <is>
-          <t>Total liabilities and shareholders’ equity</t>
-        </is>
-      </c>
-      <c r="AH38" s="3" t="n">
-        <v>323888</v>
-      </c>
-      <c r="AI38" s="3" t="n">
-        <v>338516</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4524,16 +3114,6 @@
           <t>Cash Flow Statement</t>
         </is>
       </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>Cash Flow Statement</t>
-        </is>
-      </c>
-      <c r="AG39" t="inlineStr">
-        <is>
-          <t>Cash Flow Statement</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4572,12 +3152,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="AG3:AN3"/>
     <mergeCell ref="Q3:X3"/>
     <mergeCell ref="I3:P3"/>
-    <mergeCell ref="Y3:AF3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4589,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX49"/>
+  <dimension ref="A1:AD46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4622,26 +3200,6 @@
     <col width="6" customWidth="1" min="28" max="28"/>
     <col width="6" customWidth="1" min="29" max="29"/>
     <col width="6" customWidth="1" min="30" max="30"/>
-    <col width="50" customWidth="1" min="31" max="31"/>
-    <col width="17" customWidth="1" min="32" max="32"/>
-    <col width="15" customWidth="1" min="33" max="33"/>
-    <col width="15" customWidth="1" min="34" max="34"/>
-    <col width="6" customWidth="1" min="35" max="35"/>
-    <col width="6" customWidth="1" min="36" max="36"/>
-    <col width="6" customWidth="1" min="37" max="37"/>
-    <col width="6" customWidth="1" min="38" max="38"/>
-    <col width="6" customWidth="1" min="39" max="39"/>
-    <col width="6" customWidth="1" min="40" max="40"/>
-    <col width="50" customWidth="1" min="41" max="41"/>
-    <col width="17" customWidth="1" min="42" max="42"/>
-    <col width="15" customWidth="1" min="43" max="43"/>
-    <col width="15" customWidth="1" min="44" max="44"/>
-    <col width="6" customWidth="1" min="45" max="45"/>
-    <col width="6" customWidth="1" min="46" max="46"/>
-    <col width="6" customWidth="1" min="47" max="47"/>
-    <col width="6" customWidth="1" min="48" max="48"/>
-    <col width="6" customWidth="1" min="49" max="49"/>
-    <col width="6" customWidth="1" min="50" max="50"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4668,16 +3226,6 @@
           <t>Year 2022</t>
         </is>
       </c>
-      <c r="AE3" s="2" t="inlineStr">
-        <is>
-          <t>Year 2021</t>
-        </is>
-      </c>
-      <c r="AO3" s="2" t="inlineStr">
-        <is>
-          <t>Year 2020</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4722,34 +3270,6 @@
       <c r="X4" t="n">
         <v/>
       </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Cash Flow Statement</t>
-        </is>
-      </c>
-      <c r="AF4" t="n">
-        <v/>
-      </c>
-      <c r="AG4" t="n">
-        <v/>
-      </c>
-      <c r="AH4" t="n">
-        <v/>
-      </c>
-      <c r="AO4" t="inlineStr">
-        <is>
-          <t>Cash Flow Statement</t>
-        </is>
-      </c>
-      <c r="AP4" t="n">
-        <v/>
-      </c>
-      <c r="AQ4" t="n">
-        <v/>
-      </c>
-      <c r="AR4" t="n">
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4798,38 +3318,6 @@
         <v/>
       </c>
       <c r="X5" t="n">
-        <v/>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED STATEMENTS OF CASH FLOWS - USD ($) $ in Millions</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>12 Months Ended</t>
-        </is>
-      </c>
-      <c r="AG5" t="n">
-        <v/>
-      </c>
-      <c r="AH5" t="n">
-        <v/>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>CONSOLIDATED STATEMENTS OF CASH FLOWS - USD ($) $ in Millions</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>12 Months Ended</t>
-        </is>
-      </c>
-      <c r="AQ5" t="n">
-        <v/>
-      </c>
-      <c r="AR5" t="n">
         <v/>
       </c>
     </row>
@@ -4888,42 +3376,6 @@
           <t>Sep. 26, 2020</t>
         </is>
       </c>
-      <c r="AE6" t="n">
-        <v/>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>Sep. 25, 2021</t>
-        </is>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>Sep. 26, 2020</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr">
-        <is>
-          <t>Sep. 28, 2019</t>
-        </is>
-      </c>
-      <c r="AO6" t="n">
-        <v/>
-      </c>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t>Sep. 26, 2020</t>
-        </is>
-      </c>
-      <c r="AQ6" t="inlineStr">
-        <is>
-          <t>Sep. 28, 2019</t>
-        </is>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>Sep. 29, 2018</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4986,34 +3438,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>Statement of Cash Flows [Abstract]</t>
-        </is>
-      </c>
-      <c r="AF7" t="n">
-        <v/>
-      </c>
-      <c r="AG7" t="n">
-        <v/>
-      </c>
-      <c r="AH7" t="n">
-        <v/>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>Statement of Cash Flows [Abstract]</t>
-        </is>
-      </c>
-      <c r="AP7" t="n">
-        <v/>
-      </c>
-      <c r="AQ7" t="n">
-        <v/>
-      </c>
-      <c r="AR7" t="n">
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5058,34 +3482,6 @@
       <c r="X8" s="3" t="n">
         <v>50224</v>
       </c>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>Cash, cash equivalents and restricted cash, beginning balances</t>
-        </is>
-      </c>
-      <c r="AF8" s="3" t="n">
-        <v>39789</v>
-      </c>
-      <c r="AG8" s="3" t="n">
-        <v>50224</v>
-      </c>
-      <c r="AH8" s="3" t="n">
-        <v>25913</v>
-      </c>
-      <c r="AO8" t="inlineStr">
-        <is>
-          <t>Cash, cash equivalents and restricted cash, beginning balances</t>
-        </is>
-      </c>
-      <c r="AP8" s="3" t="n">
-        <v>50224</v>
-      </c>
-      <c r="AQ8" s="3" t="n">
-        <v>25913</v>
-      </c>
-      <c r="AR8" s="3" t="n">
-        <v>20289</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5148,34 +3544,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>Operating activities:</t>
-        </is>
-      </c>
-      <c r="AF9" t="n">
-        <v/>
-      </c>
-      <c r="AG9" t="n">
-        <v/>
-      </c>
-      <c r="AH9" t="n">
-        <v/>
-      </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>Operating activities:</t>
-        </is>
-      </c>
-      <c r="AP9" t="n">
-        <v/>
-      </c>
-      <c r="AQ9" t="n">
-        <v/>
-      </c>
-      <c r="AR9" t="n">
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5220,34 +3588,6 @@
       <c r="X10" s="3" t="n">
         <v>57411</v>
       </c>
-      <c r="AE10" t="inlineStr">
-        <is>
-          <t>Net income</t>
-        </is>
-      </c>
-      <c r="AF10" s="3" t="n">
-        <v>94680</v>
-      </c>
-      <c r="AG10" s="3" t="n">
-        <v>57411</v>
-      </c>
-      <c r="AH10" s="3" t="n">
-        <v>55256</v>
-      </c>
-      <c r="AO10" t="inlineStr">
-        <is>
-          <t>Net income</t>
-        </is>
-      </c>
-      <c r="AP10" s="3" t="n">
-        <v>57411</v>
-      </c>
-      <c r="AQ10" s="3" t="n">
-        <v>55256</v>
-      </c>
-      <c r="AR10" s="3" t="n">
-        <v>59531</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5310,34 +3650,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>Adjustments to reconcile net income to cash generated by operating activities:</t>
-        </is>
-      </c>
-      <c r="AF11" t="n">
-        <v/>
-      </c>
-      <c r="AG11" t="n">
-        <v/>
-      </c>
-      <c r="AH11" t="n">
-        <v/>
-      </c>
-      <c r="AO11" t="inlineStr">
-        <is>
-          <t>Adjustments to reconcile net income to cash generated by operating activities:</t>
-        </is>
-      </c>
-      <c r="AP11" t="n">
-        <v/>
-      </c>
-      <c r="AQ11" t="n">
-        <v/>
-      </c>
-      <c r="AR11" t="n">
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5382,34 +3694,6 @@
       <c r="X12" s="3" t="n">
         <v>11056</v>
       </c>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t>Depreciation and amortization</t>
-        </is>
-      </c>
-      <c r="AF12" s="3" t="n">
-        <v>11284</v>
-      </c>
-      <c r="AG12" s="3" t="n">
-        <v>11056</v>
-      </c>
-      <c r="AH12" s="3" t="n">
-        <v>12547</v>
-      </c>
-      <c r="AO12" t="inlineStr">
-        <is>
-          <t>Depreciation and amortization</t>
-        </is>
-      </c>
-      <c r="AP12" s="3" t="n">
-        <v>11056</v>
-      </c>
-      <c r="AQ12" s="3" t="n">
-        <v>12547</v>
-      </c>
-      <c r="AR12" s="3" t="n">
-        <v>10903</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5454,34 +3738,6 @@
       <c r="X13" s="3" t="n">
         <v>6829</v>
       </c>
-      <c r="AE13" t="inlineStr">
-        <is>
-          <t>Share-based compensation expense</t>
-        </is>
-      </c>
-      <c r="AF13" s="3" t="n">
-        <v>7906</v>
-      </c>
-      <c r="AG13" s="3" t="n">
-        <v>6829</v>
-      </c>
-      <c r="AH13" s="3" t="n">
-        <v>6068</v>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>Share-based compensation expense</t>
-        </is>
-      </c>
-      <c r="AP13" s="3" t="n">
-        <v>6829</v>
-      </c>
-      <c r="AQ13" s="3" t="n">
-        <v>6068</v>
-      </c>
-      <c r="AR13" s="3" t="n">
-        <v>5340</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5526,34 +3782,6 @@
       <c r="X14" s="4" t="n">
         <v>-215</v>
       </c>
-      <c r="AE14" t="inlineStr">
-        <is>
-          <t>Deferred income tax benefit</t>
-        </is>
-      </c>
-      <c r="AF14" s="3" t="n">
-        <v>-4774</v>
-      </c>
-      <c r="AG14" s="4" t="n">
-        <v>-215</v>
-      </c>
-      <c r="AH14" s="4" t="n">
-        <v>-340</v>
-      </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t>Deferred income tax benefit</t>
-        </is>
-      </c>
-      <c r="AP14" s="4" t="n">
-        <v>-215</v>
-      </c>
-      <c r="AQ14" s="4" t="n">
-        <v>-340</v>
-      </c>
-      <c r="AR14" s="3" t="n">
-        <v>-32590</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5610,34 +3838,6 @@
       <c r="X15" s="4" t="n">
         <v>-97</v>
       </c>
-      <c r="AE15" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="AF15" s="4" t="n">
-        <v>-147</v>
-      </c>
-      <c r="AG15" s="4" t="n">
-        <v>-97</v>
-      </c>
-      <c r="AH15" s="4" t="n">
-        <v>-652</v>
-      </c>
-      <c r="AO15" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="AP15" s="4" t="n">
-        <v>-97</v>
-      </c>
-      <c r="AQ15" s="4" t="n">
-        <v>-652</v>
-      </c>
-      <c r="AR15" s="4" t="n">
-        <v>-444</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5688,34 +3888,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="AE16" t="inlineStr">
-        <is>
-          <t>Changes in operating assets and liabilities:</t>
-        </is>
-      </c>
-      <c r="AF16" t="n">
-        <v/>
-      </c>
-      <c r="AG16" t="n">
-        <v/>
-      </c>
-      <c r="AH16" t="n">
-        <v/>
-      </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>Changes in operating assets and liabilities:</t>
-        </is>
-      </c>
-      <c r="AP16" t="n">
-        <v/>
-      </c>
-      <c r="AQ16" t="n">
-        <v/>
-      </c>
-      <c r="AR16" t="n">
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5760,34 +3932,6 @@
       <c r="X17" s="3" t="n">
         <v>6917</v>
       </c>
-      <c r="AE17" t="inlineStr">
-        <is>
-          <t>Accounts receivable, net</t>
-        </is>
-      </c>
-      <c r="AF17" s="3" t="n">
-        <v>-10125</v>
-      </c>
-      <c r="AG17" s="3" t="n">
-        <v>6917</v>
-      </c>
-      <c r="AH17" s="4" t="n">
-        <v>245</v>
-      </c>
-      <c r="AO17" t="inlineStr">
-        <is>
-          <t>Accounts receivable, net</t>
-        </is>
-      </c>
-      <c r="AP17" s="3" t="n">
-        <v>6917</v>
-      </c>
-      <c r="AQ17" s="4" t="n">
-        <v>245</v>
-      </c>
-      <c r="AR17" s="3" t="n">
-        <v>-5322</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5832,34 +3976,6 @@
       <c r="X18" s="4" t="n">
         <v>-127</v>
       </c>
-      <c r="AE18" t="inlineStr">
-        <is>
-          <t>Inventories</t>
-        </is>
-      </c>
-      <c r="AF18" s="3" t="n">
-        <v>-2642</v>
-      </c>
-      <c r="AG18" s="4" t="n">
-        <v>-127</v>
-      </c>
-      <c r="AH18" s="4" t="n">
-        <v>-289</v>
-      </c>
-      <c r="AO18" t="inlineStr">
-        <is>
-          <t>Inventories</t>
-        </is>
-      </c>
-      <c r="AP18" s="4" t="n">
-        <v>-127</v>
-      </c>
-      <c r="AQ18" s="4" t="n">
-        <v>-289</v>
-      </c>
-      <c r="AR18" s="4" t="n">
-        <v>828</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5904,34 +4020,6 @@
       <c r="X19" s="3" t="n">
         <v>1553</v>
       </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>Vendor non-trade receivables</t>
-        </is>
-      </c>
-      <c r="AF19" s="3" t="n">
-        <v>-3903</v>
-      </c>
-      <c r="AG19" s="3" t="n">
-        <v>1553</v>
-      </c>
-      <c r="AH19" s="3" t="n">
-        <v>2931</v>
-      </c>
-      <c r="AO19" t="inlineStr">
-        <is>
-          <t>Vendor non-trade receivables</t>
-        </is>
-      </c>
-      <c r="AP19" s="3" t="n">
-        <v>1553</v>
-      </c>
-      <c r="AQ19" s="3" t="n">
-        <v>2931</v>
-      </c>
-      <c r="AR19" s="3" t="n">
-        <v>-8010</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5976,34 +4064,6 @@
       <c r="X20" s="3" t="n">
         <v>-9588</v>
       </c>
-      <c r="AE20" t="inlineStr">
-        <is>
-          <t>Other current and non-current assets</t>
-        </is>
-      </c>
-      <c r="AF20" s="3" t="n">
-        <v>-8042</v>
-      </c>
-      <c r="AG20" s="3" t="n">
-        <v>-9588</v>
-      </c>
-      <c r="AH20" s="4" t="n">
-        <v>873</v>
-      </c>
-      <c r="AO20" t="inlineStr">
-        <is>
-          <t>Other current and non-current assets</t>
-        </is>
-      </c>
-      <c r="AP20" s="3" t="n">
-        <v>-9588</v>
-      </c>
-      <c r="AQ20" s="4" t="n">
-        <v>873</v>
-      </c>
-      <c r="AR20" s="4" t="n">
-        <v>-423</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6048,34 +4108,6 @@
       <c r="X21" s="3" t="n">
         <v>-4062</v>
       </c>
-      <c r="AE21" t="inlineStr">
-        <is>
-          <t>Accounts payable</t>
-        </is>
-      </c>
-      <c r="AF21" s="3" t="n">
-        <v>12326</v>
-      </c>
-      <c r="AG21" s="3" t="n">
-        <v>-4062</v>
-      </c>
-      <c r="AH21" s="3" t="n">
-        <v>-1923</v>
-      </c>
-      <c r="AO21" t="inlineStr">
-        <is>
-          <t>Accounts payable</t>
-        </is>
-      </c>
-      <c r="AP21" s="3" t="n">
-        <v>-4062</v>
-      </c>
-      <c r="AQ21" s="3" t="n">
-        <v>-1923</v>
-      </c>
-      <c r="AR21" s="3" t="n">
-        <v>9175</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6120,34 +4152,6 @@
       <c r="X22" s="3" t="n">
         <v>2081</v>
       </c>
-      <c r="AE22" t="inlineStr">
-        <is>
-          <t>Deferred revenue</t>
-        </is>
-      </c>
-      <c r="AF22" s="3" t="n">
-        <v>1676</v>
-      </c>
-      <c r="AG22" s="3" t="n">
-        <v>2081</v>
-      </c>
-      <c r="AH22" s="4" t="n">
-        <v>-625</v>
-      </c>
-      <c r="AO22" t="inlineStr">
-        <is>
-          <t>Deferred revenue</t>
-        </is>
-      </c>
-      <c r="AP22" s="3" t="n">
-        <v>2081</v>
-      </c>
-      <c r="AQ22" s="4" t="n">
-        <v>-625</v>
-      </c>
-      <c r="AR22" s="4" t="n">
-        <v>-3</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6204,34 +4208,6 @@
       <c r="X23" s="3" t="n">
         <v>8916</v>
       </c>
-      <c r="AE23" t="inlineStr">
-        <is>
-          <t>Other current and non-current liabilities</t>
-        </is>
-      </c>
-      <c r="AF23" s="3" t="n">
-        <v>5799</v>
-      </c>
-      <c r="AG23" s="3" t="n">
-        <v>8916</v>
-      </c>
-      <c r="AH23" s="3" t="n">
-        <v>-4700</v>
-      </c>
-      <c r="AO23" t="inlineStr">
-        <is>
-          <t>Other current and non-current liabilities</t>
-        </is>
-      </c>
-      <c r="AP23" s="3" t="n">
-        <v>8916</v>
-      </c>
-      <c r="AQ23" s="3" t="n">
-        <v>-4700</v>
-      </c>
-      <c r="AR23" s="3" t="n">
-        <v>38449</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6276,34 +4252,6 @@
       <c r="X24" s="3" t="n">
         <v>80674</v>
       </c>
-      <c r="AE24" t="inlineStr">
-        <is>
-          <t>Cash generated by operating activities</t>
-        </is>
-      </c>
-      <c r="AF24" s="3" t="n">
-        <v>104038</v>
-      </c>
-      <c r="AG24" s="3" t="n">
-        <v>80674</v>
-      </c>
-      <c r="AH24" s="3" t="n">
-        <v>69391</v>
-      </c>
-      <c r="AO24" t="inlineStr">
-        <is>
-          <t>Cash generated by operating activities</t>
-        </is>
-      </c>
-      <c r="AP24" s="3" t="n">
-        <v>80674</v>
-      </c>
-      <c r="AQ24" s="3" t="n">
-        <v>69391</v>
-      </c>
-      <c r="AR24" s="3" t="n">
-        <v>77434</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6354,34 +4302,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="AE25" t="inlineStr">
-        <is>
-          <t>Investing activities:</t>
-        </is>
-      </c>
-      <c r="AF25" t="n">
-        <v/>
-      </c>
-      <c r="AG25" t="n">
-        <v/>
-      </c>
-      <c r="AH25" t="n">
-        <v/>
-      </c>
-      <c r="AO25" t="inlineStr">
-        <is>
-          <t>Investing activities:</t>
-        </is>
-      </c>
-      <c r="AP25" t="n">
-        <v/>
-      </c>
-      <c r="AQ25" t="n">
-        <v/>
-      </c>
-      <c r="AR25" t="n">
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6426,34 +4346,6 @@
       <c r="X26" s="3" t="n">
         <v>-114938</v>
       </c>
-      <c r="AE26" t="inlineStr">
-        <is>
-          <t>Purchases of marketable securities</t>
-        </is>
-      </c>
-      <c r="AF26" s="3" t="n">
-        <v>-109558</v>
-      </c>
-      <c r="AG26" s="3" t="n">
-        <v>-114938</v>
-      </c>
-      <c r="AH26" s="3" t="n">
-        <v>-39630</v>
-      </c>
-      <c r="AO26" t="inlineStr">
-        <is>
-          <t>Purchases of marketable securities</t>
-        </is>
-      </c>
-      <c r="AP26" s="3" t="n">
-        <v>-114938</v>
-      </c>
-      <c r="AQ26" s="3" t="n">
-        <v>-39630</v>
-      </c>
-      <c r="AR26" s="3" t="n">
-        <v>-71356</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6498,34 +4390,6 @@
       <c r="X27" s="3" t="n">
         <v>69918</v>
       </c>
-      <c r="AE27" t="inlineStr">
-        <is>
-          <t>Proceeds from maturities of marketable securities</t>
-        </is>
-      </c>
-      <c r="AF27" s="3" t="n">
-        <v>59023</v>
-      </c>
-      <c r="AG27" s="3" t="n">
-        <v>69918</v>
-      </c>
-      <c r="AH27" s="3" t="n">
-        <v>40102</v>
-      </c>
-      <c r="AO27" t="inlineStr">
-        <is>
-          <t>Proceeds from maturities of marketable securities</t>
-        </is>
-      </c>
-      <c r="AP27" s="3" t="n">
-        <v>69918</v>
-      </c>
-      <c r="AQ27" s="3" t="n">
-        <v>40102</v>
-      </c>
-      <c r="AR27" s="3" t="n">
-        <v>55881</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6570,34 +4434,6 @@
       <c r="X28" s="3" t="n">
         <v>50473</v>
       </c>
-      <c r="AE28" t="inlineStr">
-        <is>
-          <t>Proceeds from sales of marketable securities</t>
-        </is>
-      </c>
-      <c r="AF28" s="3" t="n">
-        <v>47460</v>
-      </c>
-      <c r="AG28" s="3" t="n">
-        <v>50473</v>
-      </c>
-      <c r="AH28" s="3" t="n">
-        <v>56988</v>
-      </c>
-      <c r="AO28" t="inlineStr">
-        <is>
-          <t>Proceeds from sales of marketable securities</t>
-        </is>
-      </c>
-      <c r="AP28" s="3" t="n">
-        <v>50473</v>
-      </c>
-      <c r="AQ28" s="3" t="n">
-        <v>56988</v>
-      </c>
-      <c r="AR28" s="3" t="n">
-        <v>47838</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6642,34 +4478,6 @@
       <c r="X29" s="3" t="n">
         <v>-7309</v>
       </c>
-      <c r="AE29" t="inlineStr">
-        <is>
-          <t>Payments for acquisition of property, plant and equipment</t>
-        </is>
-      </c>
-      <c r="AF29" s="3" t="n">
-        <v>-11085</v>
-      </c>
-      <c r="AG29" s="3" t="n">
-        <v>-7309</v>
-      </c>
-      <c r="AH29" s="3" t="n">
-        <v>-10495</v>
-      </c>
-      <c r="AO29" t="inlineStr">
-        <is>
-          <t>Payments for acquisition of property, plant and equipment</t>
-        </is>
-      </c>
-      <c r="AP29" s="3" t="n">
-        <v>-7309</v>
-      </c>
-      <c r="AQ29" s="3" t="n">
-        <v>-10495</v>
-      </c>
-      <c r="AR29" s="3" t="n">
-        <v>-13313</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6726,34 +4534,6 @@
       <c r="X30" s="3" t="n">
         <v>-1524</v>
       </c>
-      <c r="AE30" t="inlineStr">
-        <is>
-          <t>Payments made in connection with business acquisitions, net</t>
-        </is>
-      </c>
-      <c r="AF30" s="4" t="n">
-        <v>-33</v>
-      </c>
-      <c r="AG30" s="3" t="n">
-        <v>-1524</v>
-      </c>
-      <c r="AH30" s="4" t="n">
-        <v>-624</v>
-      </c>
-      <c r="AO30" t="inlineStr">
-        <is>
-          <t>Payments made in connection with business acquisitions, net</t>
-        </is>
-      </c>
-      <c r="AP30" s="3" t="n">
-        <v>-1524</v>
-      </c>
-      <c r="AQ30" s="4" t="n">
-        <v>-624</v>
-      </c>
-      <c r="AR30" s="4" t="n">
-        <v>-721</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6798,34 +4578,6 @@
       <c r="X31" s="4" t="n">
         <v>-909</v>
       </c>
-      <c r="AE31" t="inlineStr">
-        <is>
-          <t>Purchases of non-marketable securities</t>
-        </is>
-      </c>
-      <c r="AF31" s="4" t="n">
-        <v>-131</v>
-      </c>
-      <c r="AG31" s="4" t="n">
-        <v>-210</v>
-      </c>
-      <c r="AH31" s="3" t="n">
-        <v>-1001</v>
-      </c>
-      <c r="AO31" t="inlineStr">
-        <is>
-          <t>Purchases of non-marketable securities</t>
-        </is>
-      </c>
-      <c r="AP31" s="4" t="n">
-        <v>-210</v>
-      </c>
-      <c r="AQ31" s="3" t="n">
-        <v>-1001</v>
-      </c>
-      <c r="AR31" s="3" t="n">
-        <v>-1871</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6870,34 +4622,6 @@
       <c r="X32" s="3" t="n">
         <v>-4289</v>
       </c>
-      <c r="AE32" t="inlineStr">
-        <is>
-          <t>Proceeds from non-marketable securities</t>
-        </is>
-      </c>
-      <c r="AF32" s="4" t="n">
-        <v>387</v>
-      </c>
-      <c r="AG32" s="4" t="n">
-        <v>92</v>
-      </c>
-      <c r="AH32" s="3" t="n">
-        <v>1634</v>
-      </c>
-      <c r="AO32" t="inlineStr">
-        <is>
-          <t>Proceeds from non-marketable securities</t>
-        </is>
-      </c>
-      <c r="AP32" s="4" t="n">
-        <v>92</v>
-      </c>
-      <c r="AQ32" s="3" t="n">
-        <v>1634</v>
-      </c>
-      <c r="AR32" s="4" t="n">
-        <v>353</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6948,34 +4672,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="AE33" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="AF33" s="4" t="n">
-        <v>-608</v>
-      </c>
-      <c r="AG33" s="4" t="n">
-        <v>-791</v>
-      </c>
-      <c r="AH33" s="3" t="n">
-        <v>-1078</v>
-      </c>
-      <c r="AO33" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="AP33" s="4" t="n">
-        <v>-791</v>
-      </c>
-      <c r="AQ33" s="3" t="n">
-        <v>-1078</v>
-      </c>
-      <c r="AR33" s="4" t="n">
-        <v>-745</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7020,34 +4716,6 @@
       <c r="X34" s="3" t="n">
         <v>-3634</v>
       </c>
-      <c r="AE34" t="inlineStr">
-        <is>
-          <t>Cash generated by/(used in) investing activities</t>
-        </is>
-      </c>
-      <c r="AF34" s="3" t="n">
-        <v>-14545</v>
-      </c>
-      <c r="AG34" s="3" t="n">
-        <v>-4289</v>
-      </c>
-      <c r="AH34" s="3" t="n">
-        <v>45896</v>
-      </c>
-      <c r="AO34" t="inlineStr">
-        <is>
-          <t>Cash generated by/(used in) investing activities</t>
-        </is>
-      </c>
-      <c r="AP34" s="3" t="n">
-        <v>-4289</v>
-      </c>
-      <c r="AQ34" s="3" t="n">
-        <v>45896</v>
-      </c>
-      <c r="AR34" s="3" t="n">
-        <v>16066</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7092,34 +4760,6 @@
       <c r="X35" s="3" t="n">
         <v>-14081</v>
       </c>
-      <c r="AE35" t="inlineStr">
-        <is>
-          <t>Financing activities:</t>
-        </is>
-      </c>
-      <c r="AF35" t="n">
-        <v/>
-      </c>
-      <c r="AG35" t="n">
-        <v/>
-      </c>
-      <c r="AH35" t="n">
-        <v/>
-      </c>
-      <c r="AO35" t="inlineStr">
-        <is>
-          <t>Financing activities:</t>
-        </is>
-      </c>
-      <c r="AP35" t="n">
-        <v/>
-      </c>
-      <c r="AQ35" t="n">
-        <v/>
-      </c>
-      <c r="AR35" t="n">
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7164,34 +4804,6 @@
       <c r="X36" s="3" t="n">
         <v>-72358</v>
       </c>
-      <c r="AE36" t="inlineStr">
-        <is>
-          <t>Proceeds from issuance of common stock</t>
-        </is>
-      </c>
-      <c r="AF36" s="3" t="n">
-        <v>1105</v>
-      </c>
-      <c r="AG36" s="4" t="n">
-        <v>880</v>
-      </c>
-      <c r="AH36" s="4" t="n">
-        <v>781</v>
-      </c>
-      <c r="AO36" t="inlineStr">
-        <is>
-          <t>Proceeds from issuance of common stock</t>
-        </is>
-      </c>
-      <c r="AP36" s="4" t="n">
-        <v>880</v>
-      </c>
-      <c r="AQ36" s="4" t="n">
-        <v>781</v>
-      </c>
-      <c r="AR36" s="4" t="n">
-        <v>669</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7236,34 +4848,6 @@
       <c r="X37" s="3" t="n">
         <v>16091</v>
       </c>
-      <c r="AE37" t="inlineStr">
-        <is>
-          <t>Payments for taxes related to net share settlement of equity awards</t>
-        </is>
-      </c>
-      <c r="AF37" s="3" t="n">
-        <v>-6556</v>
-      </c>
-      <c r="AG37" s="3" t="n">
-        <v>-3634</v>
-      </c>
-      <c r="AH37" s="3" t="n">
-        <v>-2817</v>
-      </c>
-      <c r="AO37" t="inlineStr">
-        <is>
-          <t>Payments for taxes related to net share settlement of equity awards</t>
-        </is>
-      </c>
-      <c r="AP37" s="3" t="n">
-        <v>-3634</v>
-      </c>
-      <c r="AQ37" s="3" t="n">
-        <v>-2817</v>
-      </c>
-      <c r="AR37" s="3" t="n">
-        <v>-2527</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7308,34 +4892,6 @@
       <c r="X38" s="3" t="n">
         <v>-12629</v>
       </c>
-      <c r="AE38" t="inlineStr">
-        <is>
-          <t>Payments for dividends and dividend equivalents</t>
-        </is>
-      </c>
-      <c r="AF38" s="3" t="n">
-        <v>-14467</v>
-      </c>
-      <c r="AG38" s="3" t="n">
-        <v>-14081</v>
-      </c>
-      <c r="AH38" s="3" t="n">
-        <v>-14119</v>
-      </c>
-      <c r="AO38" t="inlineStr">
-        <is>
-          <t>Payments for dividends and dividend equivalents</t>
-        </is>
-      </c>
-      <c r="AP38" s="3" t="n">
-        <v>-14081</v>
-      </c>
-      <c r="AQ38" s="3" t="n">
-        <v>-14119</v>
-      </c>
-      <c r="AR38" s="3" t="n">
-        <v>-13712</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7380,34 +4936,6 @@
       <c r="X39" s="4" t="n">
         <v>-963</v>
       </c>
-      <c r="AE39" t="inlineStr">
-        <is>
-          <t>Repurchases of common stock</t>
-        </is>
-      </c>
-      <c r="AF39" s="3" t="n">
-        <v>-85971</v>
-      </c>
-      <c r="AG39" s="3" t="n">
-        <v>-72358</v>
-      </c>
-      <c r="AH39" s="3" t="n">
-        <v>-66897</v>
-      </c>
-      <c r="AO39" t="inlineStr">
-        <is>
-          <t>Repurchases of common stock</t>
-        </is>
-      </c>
-      <c r="AP39" s="3" t="n">
-        <v>-72358</v>
-      </c>
-      <c r="AQ39" s="3" t="n">
-        <v>-66897</v>
-      </c>
-      <c r="AR39" s="3" t="n">
-        <v>-72738</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7452,34 +4980,6 @@
       <c r="X40" s="4" t="n">
         <v>754</v>
       </c>
-      <c r="AE40" t="inlineStr">
-        <is>
-          <t>Proceeds from issuance of term debt, net</t>
-        </is>
-      </c>
-      <c r="AF40" s="3" t="n">
-        <v>20393</v>
-      </c>
-      <c r="AG40" s="3" t="n">
-        <v>16091</v>
-      </c>
-      <c r="AH40" s="3" t="n">
-        <v>6963</v>
-      </c>
-      <c r="AO40" t="inlineStr">
-        <is>
-          <t>Proceeds from issuance of term debt, net</t>
-        </is>
-      </c>
-      <c r="AP40" s="3" t="n">
-        <v>16091</v>
-      </c>
-      <c r="AQ40" s="3" t="n">
-        <v>6963</v>
-      </c>
-      <c r="AR40" s="3" t="n">
-        <v>6969</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -7536,34 +5036,6 @@
       <c r="X41" s="3" t="n">
         <v>-86820</v>
       </c>
-      <c r="AE41" t="inlineStr">
-        <is>
-          <t>Repayments of term debt</t>
-        </is>
-      </c>
-      <c r="AF41" s="3" t="n">
-        <v>-8750</v>
-      </c>
-      <c r="AG41" s="3" t="n">
-        <v>-12629</v>
-      </c>
-      <c r="AH41" s="3" t="n">
-        <v>-8805</v>
-      </c>
-      <c r="AO41" t="inlineStr">
-        <is>
-          <t>Repayments of term debt</t>
-        </is>
-      </c>
-      <c r="AP41" s="3" t="n">
-        <v>-12629</v>
-      </c>
-      <c r="AQ41" s="3" t="n">
-        <v>-8805</v>
-      </c>
-      <c r="AR41" s="3" t="n">
-        <v>-6500</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -7608,34 +5080,6 @@
       <c r="X42" s="3" t="n">
         <v>-10435</v>
       </c>
-      <c r="AE42" t="inlineStr">
-        <is>
-          <t>Proceeds from/(Repayments of) commercial paper, net</t>
-        </is>
-      </c>
-      <c r="AF42" s="3" t="n">
-        <v>1022</v>
-      </c>
-      <c r="AG42" s="4" t="n">
-        <v>-963</v>
-      </c>
-      <c r="AH42" s="3" t="n">
-        <v>-5977</v>
-      </c>
-      <c r="AO42" t="inlineStr">
-        <is>
-          <t>Repayments of commercial paper, net</t>
-        </is>
-      </c>
-      <c r="AP42" s="4" t="n">
-        <v>-963</v>
-      </c>
-      <c r="AQ42" s="3" t="n">
-        <v>-5977</v>
-      </c>
-      <c r="AR42" s="4" t="n">
-        <v>-37</v>
-      </c>
     </row>
     <row r="43">
       <c r="K43" t="inlineStr">
@@ -7666,34 +5110,6 @@
       <c r="X43" s="3" t="n">
         <v>39789</v>
       </c>
-      <c r="AE43" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="AF43" s="4" t="n">
-        <v>-129</v>
-      </c>
-      <c r="AG43" s="4" t="n">
-        <v>-126</v>
-      </c>
-      <c r="AH43" s="4" t="n">
-        <v>-105</v>
-      </c>
-      <c r="AO43" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="AP43" s="4" t="n">
-        <v>-126</v>
-      </c>
-      <c r="AQ43" s="4" t="n">
-        <v>-105</v>
-      </c>
-      <c r="AR43" s="4" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="44">
       <c r="U44" t="inlineStr">
@@ -7716,34 +5132,6 @@
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="AE44" t="inlineStr">
-        <is>
-          <t>Cash used in financing activities</t>
-        </is>
-      </c>
-      <c r="AF44" s="3" t="n">
-        <v>-93353</v>
-      </c>
-      <c r="AG44" s="3" t="n">
-        <v>-86820</v>
-      </c>
-      <c r="AH44" s="3" t="n">
-        <v>-90976</v>
-      </c>
-      <c r="AO44" t="inlineStr">
-        <is>
-          <t>Cash used in financing activities</t>
-        </is>
-      </c>
-      <c r="AP44" s="3" t="n">
-        <v>-86820</v>
-      </c>
-      <c r="AQ44" s="3" t="n">
-        <v>-90976</v>
-      </c>
-      <c r="AR44" s="3" t="n">
-        <v>-87876</v>
-      </c>
     </row>
     <row r="45">
       <c r="U45" t="inlineStr">
@@ -7760,34 +5148,6 @@
       <c r="X45" s="3" t="n">
         <v>9501</v>
       </c>
-      <c r="AE45" t="inlineStr">
-        <is>
-          <t>Increase/(Decrease) in cash, cash equivalents and restricted cash</t>
-        </is>
-      </c>
-      <c r="AF45" s="3" t="n">
-        <v>-3860</v>
-      </c>
-      <c r="AG45" s="3" t="n">
-        <v>-10435</v>
-      </c>
-      <c r="AH45" s="3" t="n">
-        <v>24311</v>
-      </c>
-      <c r="AO45" t="inlineStr">
-        <is>
-          <t>Increase/(Decrease) in cash, cash equivalents and restricted cash</t>
-        </is>
-      </c>
-      <c r="AP45" s="3" t="n">
-        <v>-10435</v>
-      </c>
-      <c r="AQ45" s="3" t="n">
-        <v>24311</v>
-      </c>
-      <c r="AR45" s="3" t="n">
-        <v>5624</v>
-      </c>
     </row>
     <row r="46">
       <c r="U46" t="inlineStr">
@@ -7804,132 +5164,12 @@
       <c r="X46" s="3" t="n">
         <v>3002</v>
       </c>
-      <c r="AE46" t="inlineStr">
-        <is>
-          <t>Cash, cash equivalents and restricted cash, ending balances</t>
-        </is>
-      </c>
-      <c r="AF46" s="3" t="n">
-        <v>35929</v>
-      </c>
-      <c r="AG46" s="3" t="n">
-        <v>39789</v>
-      </c>
-      <c r="AH46" s="3" t="n">
-        <v>50224</v>
-      </c>
-      <c r="AO46" t="inlineStr">
-        <is>
-          <t>Cash, cash equivalents and restricted cash, ending balances</t>
-        </is>
-      </c>
-      <c r="AP46" s="3" t="n">
-        <v>39789</v>
-      </c>
-      <c r="AQ46" s="3" t="n">
-        <v>50224</v>
-      </c>
-      <c r="AR46" s="3" t="n">
-        <v>25913</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="AE47" t="inlineStr">
-        <is>
-          <t>Supplemental cash flow disclosure:</t>
-        </is>
-      </c>
-      <c r="AF47" t="n">
-        <v/>
-      </c>
-      <c r="AG47" t="n">
-        <v/>
-      </c>
-      <c r="AH47" t="n">
-        <v/>
-      </c>
-      <c r="AO47" t="inlineStr">
-        <is>
-          <t>Supplemental cash flow disclosure:</t>
-        </is>
-      </c>
-      <c r="AP47" t="n">
-        <v/>
-      </c>
-      <c r="AQ47" t="n">
-        <v/>
-      </c>
-      <c r="AR47" t="n">
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="AE48" t="inlineStr">
-        <is>
-          <t>Cash paid for income taxes, net</t>
-        </is>
-      </c>
-      <c r="AF48" s="3" t="n">
-        <v>25385</v>
-      </c>
-      <c r="AG48" s="3" t="n">
-        <v>9501</v>
-      </c>
-      <c r="AH48" s="3" t="n">
-        <v>15263</v>
-      </c>
-      <c r="AO48" t="inlineStr">
-        <is>
-          <t>Cash paid for income taxes, net</t>
-        </is>
-      </c>
-      <c r="AP48" s="3" t="n">
-        <v>9501</v>
-      </c>
-      <c r="AQ48" s="3" t="n">
-        <v>15263</v>
-      </c>
-      <c r="AR48" s="3" t="n">
-        <v>10417</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="AE49" t="inlineStr">
-        <is>
-          <t>Cash paid for interest</t>
-        </is>
-      </c>
-      <c r="AF49" s="3" t="n">
-        <v>2687</v>
-      </c>
-      <c r="AG49" s="3" t="n">
-        <v>3002</v>
-      </c>
-      <c r="AH49" s="3" t="n">
-        <v>3423</v>
-      </c>
-      <c r="AO49" t="inlineStr">
-        <is>
-          <t>Cash paid for interest</t>
-        </is>
-      </c>
-      <c r="AP49" s="3" t="n">
-        <v>3002</v>
-      </c>
-      <c r="AQ49" s="3" t="n">
-        <v>3423</v>
-      </c>
-      <c r="AR49" s="3" t="n">
-        <v>3022</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A3:J3"/>
+  <mergeCells count="3">
     <mergeCell ref="K3:T3"/>
     <mergeCell ref="U3:AD3"/>
-    <mergeCell ref="AO3:AX3"/>
-    <mergeCell ref="AE3:AN3"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>